<commit_message>
chore(examples): regenerate stale team-formula xlsx (whitespace-only)
The 6 example files committed in 1237c09 ("fix(helper): team PW/PL
sum all sub-bouts in Google Sheets / Apple Numbers") carry extra
whitespace inside the team-formula expressions:

  IF(UPPER(D5)="X",0,IF((LEN(...)) +LEN(...)) )>(LEN(...)) +LEN(...)) ),1,0))

while the committed Go code in buildTeamWinnersFormula already used
fmt.Sprintf("(%s+%s)", ...) — i.e. no spaces. The likely cause is
that `make examples` was run against an intermediate draft of the
formula builder that included spaces; the builder was tidied to the
no-space form before commit, but the xlsx files were not regenerated.

Regenerated with `make examples`; output is functionally identical
(Excel ignores whitespace around operators), just no longer stale
against the current generator.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/playoffs-example-small.xlsx
+++ b/playoffs-example-small.xlsx
@@ -1289,17 +1289,17 @@
         <v>37</v>
       </c>
       <c r="B12" s="19" t="str">
-        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C12" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D12" s="19"/>
       <c r="E12" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F12" s="19" t="str">
-        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G12" s="19" t="s">
         <v>37</v>
@@ -1443,17 +1443,17 @@
         <v>37</v>
       </c>
       <c r="B28" s="19" t="str">
-        <f>IF(UPPER(D21)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D22)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D23)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D24)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D25)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D21)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D22)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D23)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D24)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D25)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C28" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D28" s="19"/>
       <c r="E28" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F28" s="19" t="str">
-        <f>IF(UPPER(D21)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D22)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D23)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D24)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D25)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D21)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D22)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D23)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D24)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D25)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G28" s="19" t="s">
         <v>37</v>
@@ -1597,17 +1597,17 @@
         <v>37</v>
       </c>
       <c r="B49" s="19" t="str">
-        <f>IF(UPPER(D42)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C42," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F42," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D43)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C43," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F43," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D44)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C44," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F44," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D45)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C45," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F45," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D46)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C46," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E46," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F46," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D42)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C42," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F42," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D43)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C43," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F43," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D44)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C44," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F44," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D45)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C45," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F45," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D46)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C46," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E46," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F46," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C49" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C46," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C46," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D49" s="19"/>
       <c r="E49" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E46," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F46," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E46," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F46," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F49" s="19" t="str">
-        <f>IF(UPPER(D42)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F42," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B42," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C42," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D43)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F43," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C43," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D44)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F44," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B44," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C44," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D45)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F45," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B45," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C45," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D46)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E46," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F46," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C46," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D42)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F42," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B42," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C42," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D43)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F43," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C43," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D44)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F44," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B44," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C44," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D45)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F45," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B45," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C45," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D46)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E46," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F46," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C46," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G49" s="19" t="s">
         <v>37</v>
@@ -1751,17 +1751,17 @@
         <v>37</v>
       </c>
       <c r="B65" s="19" t="str">
-        <f>IF(UPPER(D58)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C58," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F58," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D59)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C59," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F59," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D60)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C60," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F60," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D61)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C61," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F61," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D62)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C62," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E62," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F62," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D58)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C58," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F58," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D59)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C59," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F59," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D60)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C60," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F60," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D61)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C61," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F61," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D62)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C62," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E62," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F62," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C65" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C62," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C62," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D65" s="19"/>
       <c r="E65" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E62," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F62," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E62," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F62," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F65" s="19" t="str">
-        <f>IF(UPPER(D58)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F58," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B58," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C58," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D59)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F59," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B59," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C59," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D60)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F60," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B60," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C60," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D61)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F61," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B61," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C61," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D62)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E62," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F62," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C62," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D58)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F58," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B58," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C58," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D59)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F59," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B59," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C59," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D60)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F60," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B60," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C60," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D61)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F61," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B61," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C61," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D62)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E62," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F62," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C62," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G65" s="19" t="s">
         <v>37</v>
@@ -1905,17 +1905,17 @@
         <v>37</v>
       </c>
       <c r="B81" s="19" t="str">
-        <f>IF(UPPER(D74)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C74," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F74," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D75)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C75," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F75," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D76)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C76," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F76," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D77)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C77," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F77," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D78)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B78," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C78," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E78," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F78," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D74)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C74," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F74," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D75)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C75," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F75," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D76)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C76," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F76," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D77)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C77," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F77," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D78)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B78," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C78," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E78," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F78," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C81" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B78," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C78," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B78," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C78," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D81" s="19"/>
       <c r="E81" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E78," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F78," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E78," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F78," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F81" s="19" t="str">
-        <f>IF(UPPER(D74)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F74," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C74," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D75)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F75," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C75," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D76)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F76," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C76," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D77)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F77," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B77," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C77," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D78)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E78," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F78," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B78," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C78," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D74)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F74," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C74," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D75)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F75," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C75," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D76)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F76," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C76," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D77)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F77," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B77," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C77," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D78)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E78," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F78," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B78," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C78," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G81" s="19" t="s">
         <v>37</v>
@@ -2059,17 +2059,17 @@
         <v>37</v>
       </c>
       <c r="B97" s="19" t="str">
-        <f>IF(UPPER(D90)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C90," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F90," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D91)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C91," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F91," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D92)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C92," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F92," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D93)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C93," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F93," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D94)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B94," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C94," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E94," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F94," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D90)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C90," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F90," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D91)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C91," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F91," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D92)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C92," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F92," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D93)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C93," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F93," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D94)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B94," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C94," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E94," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F94," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C97" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B94," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C94," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B94," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C94," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D97" s="19"/>
       <c r="E97" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E94," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F94," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E94," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F94," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F97" s="19" t="str">
-        <f>IF(UPPER(D90)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F90," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C90," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D91)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F91," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C91," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D92)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F92," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B92," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C92," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D93)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F93," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B93," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C93," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D94)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E94," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F94," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B94," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C94," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D90)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F90," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C90," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D91)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F91," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C91," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D92)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F92," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B92," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C92," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D93)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F93," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B93," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C93," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D94)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E94," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F94," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B94," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C94," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G97" s="19" t="s">
         <v>37</v>
@@ -2213,17 +2213,17 @@
         <v>37</v>
       </c>
       <c r="B118" s="19" t="str">
-        <f>IF(UPPER(D111)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C111," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F111," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D112)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C112," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F112," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D113)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C113," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F113," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D114)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C114," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F114," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D115)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B115," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C115," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E115," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F115," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D111)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C111," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F111," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D112)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C112," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F112," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D113)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C113," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F113," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D114)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C114," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F114," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D115)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B115," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C115," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E115," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F115," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C118" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B115," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C115," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B115," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C115," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D118" s="19"/>
       <c r="E118" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E115," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F115," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E115," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F115," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F118" s="19" t="str">
-        <f>IF(UPPER(D111)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F111," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B111," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C111," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D112)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F112," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B112," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C112," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D113)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F113," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B113," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C113," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D114)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F114," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B114," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C114," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D115)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E115," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F115," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B115," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C115," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D111)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F111," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B111," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C111," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D112)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F112," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B112," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C112," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D113)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F113," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B113," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C113," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D114)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F114," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B114," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C114," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D115)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E115," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F115," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B115," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C115," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G118" s="19" t="s">
         <v>37</v>
@@ -2367,17 +2367,17 @@
         <v>37</v>
       </c>
       <c r="B134" s="19" t="str">
-        <f>IF(UPPER(D127)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C127," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F127," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D128)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C128," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F128," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D129)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C129," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F129," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D130)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C130," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F130," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D131)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B131," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C131," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E131," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F131," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D127)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C127," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F127," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D128)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C128," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F128," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D129)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C129," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F129," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D130)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C130," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F130," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D131)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B131," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C131," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E131," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F131," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C134" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B131," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C131," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B131," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C131," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D134" s="19"/>
       <c r="E134" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E131," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F131," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E131," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F131," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F134" s="19" t="str">
-        <f>IF(UPPER(D127)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F127," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B127," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C127," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D128)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F128," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B128," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C128," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D129)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F129," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B129," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C129," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D130)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F130," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B130," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C130," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D131)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E131," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F131," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B131," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C131," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D127)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F127," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B127," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C127," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D128)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F128," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B128," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C128," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D129)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F129," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B129," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C129," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D130)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F130," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B130," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C130," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D131)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E131," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F131," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B131," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C131," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G134" s="19" t="s">
         <v>37</v>
@@ -2521,17 +2521,17 @@
         <v>37</v>
       </c>
       <c r="B155" s="19" t="str">
-        <f>IF(UPPER(D148)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C148," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F148," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D149)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C149," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F149," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D150)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C150," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F150," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D151)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C151," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F151," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D152)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B152," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C152," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E152," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F152," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D148)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C148," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F148," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D149)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C149," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F149," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D150)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C150," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F150," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D151)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C151," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F151," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D152)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B152," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C152," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E152," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F152," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="C155" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B152," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C152," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B152," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C152," ",""),"0",""),"-",""))</f>
       </c>
       <c r="D155" s="19"/>
       <c r="E155" s="19" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E152," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F152," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E152," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F152," ",""),"0",""),"-",""))</f>
       </c>
       <c r="F155" s="19" t="str">
-        <f>IF(UPPER(D148)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F148," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B148," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C148," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D149)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F149," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B149," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C149," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D150)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F150," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B150," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C150," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D151)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F151," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B151," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C151," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D152)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E152," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F152," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B152," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C152," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D148)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F148," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B148," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C148," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D149)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F149," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B149," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C149," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D150)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F150," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B150," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C150," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D151)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F151," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B151," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C151," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D152)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E152," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F152," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B152," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C152," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G155" s="19" t="s">
         <v>37</v>

</xml_diff>